<commit_message>
E급 = Emperor 확정, 헌제 King 지정 금지
기획자 확인 사항을 GDD에 반영했다.

- E는 D 아래 등급이 아니라 Emperor의 약자다. 등급 서열 밖의 별도 분류이며
  헌제 한 명뿐이다. SP 7은 전 등급 최고(S급 6보다 비싸다).
  능력치 1/1/1은 "「황제옹립」 하나로만 존재 가치가 성립한다"는 의도된 설계.
- 헌제의 King 지정은 금지로 확정 (§12 미결 9번 해소).
- §3.6의 「차동풍」 설명을 B3 판정에 맞게 정정 — 2회 사용이 아니라
  이미 써버린 스킬의 재활성화다.
- 엑셀 갱신 반영: 식소사번 주기 time 100 → 200.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/삼국지 약식체스.xlsx
+++ b/docs/삼국지 약식체스.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Hackers_IELTS_Listening_Basic_MP3_free\DGGL\Games\SamHero\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Samchess\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C80B1F-8566-4715-BDFC-3BEBABD2E4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9207FA55-1DDC-4B86-B19E-9564438C44C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-16320" yWindow="-16410" windowWidth="16440" windowHeight="28320" xr2:uid="{67B41BAA-AEF2-4AF0-8CD2-0E8DEEEF200D}"/>
   </bookViews>
@@ -1916,10 +1916,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>적군 1명을 지정. 그 적은 게임이 끝날 때 까지 time 100 마다 HP 1 감소</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>모든 아군이 이번 게임에서 고유 스킬을 두 번 사용할 수 있음</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1993,6 +1989,10 @@
   </si>
   <si>
     <t>적의 SP 값을 1 내린다.</t>
+  </si>
+  <si>
+    <t>적군 1명을 지정. 그 적은 게임이 끝날 때 까지 time 200 마다 HP 1 감소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2164,7 +2164,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2220,9 +2220,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2820,7 +2817,7 @@
         <v>510</v>
       </c>
       <c r="E15" t="s">
-        <v>536</v>
+        <v>557</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -2939,7 +2936,7 @@
         <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -2956,7 +2953,7 @@
         <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -3041,7 +3038,7 @@
         <v>50</v>
       </c>
       <c r="E29" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -3136,13 +3133,13 @@
       <c r="B36" t="s">
         <v>176</v>
       </c>
-      <c r="C36" s="19" t="s">
+      <c r="C36" t="s">
         <v>236</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" t="s">
         <v>237</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" t="s">
         <v>527</v>
       </c>
     </row>
@@ -3153,13 +3150,13 @@
       <c r="B37" t="s">
         <v>188</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="C37" t="s">
         <v>236</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" t="s">
         <v>237</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="E37" t="s">
         <v>527</v>
       </c>
     </row>
@@ -3170,14 +3167,14 @@
       <c r="B38" t="s">
         <v>159</v>
       </c>
-      <c r="C38" s="19" t="s">
+      <c r="C38" t="s">
         <v>236</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" t="s">
         <v>237</v>
       </c>
-      <c r="E38" s="19" t="s">
-        <v>549</v>
+      <c r="E38" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
@@ -3187,14 +3184,14 @@
       <c r="B39" t="s">
         <v>164</v>
       </c>
-      <c r="C39" s="19" t="s">
+      <c r="C39" t="s">
         <v>236</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D39" t="s">
         <v>237</v>
       </c>
-      <c r="E39" s="19" t="s">
-        <v>549</v>
+      <c r="E39" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
@@ -3204,14 +3201,14 @@
       <c r="B40" t="s">
         <v>156</v>
       </c>
-      <c r="C40" s="19" t="s">
+      <c r="C40" t="s">
         <v>236</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D40" t="s">
         <v>237</v>
       </c>
-      <c r="E40" s="19" t="s">
-        <v>549</v>
+      <c r="E40" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.45">
@@ -3221,14 +3218,14 @@
       <c r="B41" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="19" t="s">
+      <c r="C41" t="s">
         <v>236</v>
       </c>
-      <c r="D41" s="19" t="s">
+      <c r="D41" t="s">
         <v>237</v>
       </c>
-      <c r="E41" s="19" t="s">
-        <v>549</v>
+      <c r="E41" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
@@ -3238,14 +3235,14 @@
       <c r="B42" t="s">
         <v>141</v>
       </c>
-      <c r="C42" s="19" t="s">
+      <c r="C42" t="s">
         <v>236</v>
       </c>
-      <c r="D42" s="19" t="s">
+      <c r="D42" t="s">
         <v>237</v>
       </c>
-      <c r="E42" s="19" t="s">
-        <v>549</v>
+      <c r="E42" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
@@ -3255,14 +3252,14 @@
       <c r="B43" t="s">
         <v>217</v>
       </c>
-      <c r="C43" s="19" t="s">
+      <c r="C43" t="s">
         <v>236</v>
       </c>
-      <c r="D43" s="19" t="s">
+      <c r="D43" t="s">
         <v>237</v>
       </c>
-      <c r="E43" s="19" t="s">
-        <v>549</v>
+      <c r="E43" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
@@ -3272,14 +3269,14 @@
       <c r="B44" t="s">
         <v>227</v>
       </c>
-      <c r="C44" s="19" t="s">
+      <c r="C44" t="s">
         <v>236</v>
       </c>
-      <c r="D44" s="19" t="s">
+      <c r="D44" t="s">
         <v>237</v>
       </c>
-      <c r="E44" s="19" t="s">
-        <v>549</v>
+      <c r="E44" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
@@ -3289,14 +3286,14 @@
       <c r="B45" t="s">
         <v>214</v>
       </c>
-      <c r="C45" s="19" t="s">
+      <c r="C45" t="s">
         <v>236</v>
       </c>
-      <c r="D45" s="19" t="s">
+      <c r="D45" t="s">
         <v>237</v>
       </c>
-      <c r="E45" s="19" t="s">
-        <v>549</v>
+      <c r="E45" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
@@ -3306,13 +3303,13 @@
       <c r="B46" t="s">
         <v>167</v>
       </c>
-      <c r="C46" s="19" t="s">
+      <c r="C46" t="s">
         <v>238</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D46" t="s">
         <v>239</v>
       </c>
-      <c r="E46" s="19" t="s">
+      <c r="E46" t="s">
         <v>528</v>
       </c>
     </row>
@@ -3323,13 +3320,13 @@
       <c r="B47" t="s">
         <v>190</v>
       </c>
-      <c r="C47" s="19" t="s">
+      <c r="C47" t="s">
         <v>238</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D47" t="s">
         <v>239</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" t="s">
         <v>528</v>
       </c>
     </row>
@@ -3340,14 +3337,14 @@
       <c r="B48" t="s">
         <v>191</v>
       </c>
-      <c r="C48" s="19" t="s">
+      <c r="C48" t="s">
         <v>238</v>
       </c>
-      <c r="D48" s="19" t="s">
+      <c r="D48" t="s">
         <v>239</v>
       </c>
-      <c r="E48" s="19" t="s">
-        <v>550</v>
+      <c r="E48" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.45">
@@ -3357,14 +3354,14 @@
       <c r="B49" t="s">
         <v>161</v>
       </c>
-      <c r="C49" s="19" t="s">
+      <c r="C49" t="s">
         <v>238</v>
       </c>
-      <c r="D49" s="19" t="s">
+      <c r="D49" t="s">
         <v>239</v>
       </c>
-      <c r="E49" s="19" t="s">
-        <v>550</v>
+      <c r="E49" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.45">
@@ -3374,14 +3371,14 @@
       <c r="B50" t="s">
         <v>168</v>
       </c>
-      <c r="C50" s="19" t="s">
+      <c r="C50" t="s">
         <v>238</v>
       </c>
-      <c r="D50" s="19" t="s">
+      <c r="D50" t="s">
         <v>239</v>
       </c>
-      <c r="E50" s="19" t="s">
-        <v>550</v>
+      <c r="E50" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.45">
@@ -3391,14 +3388,14 @@
       <c r="B51" t="s">
         <v>142</v>
       </c>
-      <c r="C51" s="19" t="s">
+      <c r="C51" t="s">
         <v>238</v>
       </c>
-      <c r="D51" s="19" t="s">
+      <c r="D51" t="s">
         <v>239</v>
       </c>
-      <c r="E51" s="19" t="s">
-        <v>550</v>
+      <c r="E51" t="s">
+        <v>549</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.45">
@@ -3430,13 +3427,13 @@
       <c r="B54" t="s">
         <v>226</v>
       </c>
-      <c r="C54" s="19" t="s">
+      <c r="C54" t="s">
         <v>240</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D54" t="s">
         <v>241</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" t="s">
         <v>529</v>
       </c>
     </row>
@@ -3447,13 +3444,13 @@
       <c r="B55" t="s">
         <v>152</v>
       </c>
-      <c r="C55" s="19" t="s">
+      <c r="C55" t="s">
         <v>240</v>
       </c>
-      <c r="D55" s="19" t="s">
+      <c r="D55" t="s">
         <v>241</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" t="s">
         <v>529</v>
       </c>
     </row>
@@ -3464,14 +3461,14 @@
       <c r="B56" t="s">
         <v>212</v>
       </c>
-      <c r="C56" s="19" t="s">
+      <c r="C56" t="s">
         <v>240</v>
       </c>
-      <c r="D56" s="19" t="s">
+      <c r="D56" t="s">
         <v>241</v>
       </c>
-      <c r="E56" s="19" t="s">
-        <v>551</v>
+      <c r="E56" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.45">
@@ -3481,14 +3478,14 @@
       <c r="B57" t="s">
         <v>208</v>
       </c>
-      <c r="C57" s="19" t="s">
+      <c r="C57" t="s">
         <v>240</v>
       </c>
-      <c r="D57" s="19" t="s">
+      <c r="D57" t="s">
         <v>241</v>
       </c>
-      <c r="E57" s="19" t="s">
-        <v>551</v>
+      <c r="E57" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.45">
@@ -3498,14 +3495,14 @@
       <c r="B58" t="s">
         <v>163</v>
       </c>
-      <c r="C58" s="19" t="s">
+      <c r="C58" t="s">
         <v>240</v>
       </c>
-      <c r="D58" s="19" t="s">
+      <c r="D58" t="s">
         <v>241</v>
       </c>
-      <c r="E58" s="19" t="s">
-        <v>551</v>
+      <c r="E58" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.45">
@@ -3515,14 +3512,14 @@
       <c r="B59" t="s">
         <v>193</v>
       </c>
-      <c r="C59" s="19" t="s">
+      <c r="C59" t="s">
         <v>240</v>
       </c>
-      <c r="D59" s="19" t="s">
+      <c r="D59" t="s">
         <v>241</v>
       </c>
-      <c r="E59" s="19" t="s">
-        <v>551</v>
+      <c r="E59" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.45">
@@ -3532,14 +3529,14 @@
       <c r="B60" t="s">
         <v>213</v>
       </c>
-      <c r="C60" s="19" t="s">
+      <c r="C60" t="s">
         <v>240</v>
       </c>
-      <c r="D60" s="19" t="s">
+      <c r="D60" t="s">
         <v>241</v>
       </c>
-      <c r="E60" s="19" t="s">
-        <v>551</v>
+      <c r="E60" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.45">
@@ -3549,14 +3546,14 @@
       <c r="B61" t="s">
         <v>148</v>
       </c>
-      <c r="C61" s="19" t="s">
+      <c r="C61" t="s">
         <v>240</v>
       </c>
-      <c r="D61" s="19" t="s">
+      <c r="D61" t="s">
         <v>241</v>
       </c>
-      <c r="E61" s="19" t="s">
-        <v>551</v>
+      <c r="E61" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.45">
@@ -3566,14 +3563,14 @@
       <c r="B62" t="s">
         <v>189</v>
       </c>
-      <c r="C62" s="19" t="s">
+      <c r="C62" t="s">
         <v>240</v>
       </c>
-      <c r="D62" s="19" t="s">
+      <c r="D62" t="s">
         <v>241</v>
       </c>
-      <c r="E62" s="19" t="s">
-        <v>551</v>
+      <c r="E62" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.45">
@@ -3583,14 +3580,14 @@
       <c r="B63" t="s">
         <v>140</v>
       </c>
-      <c r="C63" s="19" t="s">
+      <c r="C63" t="s">
         <v>240</v>
       </c>
-      <c r="D63" s="19" t="s">
+      <c r="D63" t="s">
         <v>241</v>
       </c>
-      <c r="E63" s="19" t="s">
-        <v>551</v>
+      <c r="E63" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.45">
@@ -3600,14 +3597,14 @@
       <c r="B64" t="s">
         <v>195</v>
       </c>
-      <c r="C64" s="19" t="s">
+      <c r="C64" t="s">
         <v>240</v>
       </c>
-      <c r="D64" s="19" t="s">
+      <c r="D64" t="s">
         <v>241</v>
       </c>
-      <c r="E64" s="19" t="s">
-        <v>551</v>
+      <c r="E64" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.45">
@@ -3617,14 +3614,14 @@
       <c r="B65" t="s">
         <v>146</v>
       </c>
-      <c r="C65" s="19" t="s">
+      <c r="C65" t="s">
         <v>240</v>
       </c>
-      <c r="D65" s="19" t="s">
+      <c r="D65" t="s">
         <v>241</v>
       </c>
-      <c r="E65" s="19" t="s">
-        <v>551</v>
+      <c r="E65" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.45">
@@ -3634,14 +3631,14 @@
       <c r="B66" t="s">
         <v>145</v>
       </c>
-      <c r="C66" s="19" t="s">
+      <c r="C66" t="s">
         <v>240</v>
       </c>
-      <c r="D66" s="19" t="s">
+      <c r="D66" t="s">
         <v>241</v>
       </c>
-      <c r="E66" s="19" t="s">
-        <v>551</v>
+      <c r="E66" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.45">
@@ -3651,14 +3648,14 @@
       <c r="B67" t="s">
         <v>198</v>
       </c>
-      <c r="C67" s="19" t="s">
+      <c r="C67" t="s">
         <v>240</v>
       </c>
-      <c r="D67" s="19" t="s">
+      <c r="D67" t="s">
         <v>241</v>
       </c>
-      <c r="E67" s="19" t="s">
-        <v>551</v>
+      <c r="E67" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.45">
@@ -3668,13 +3665,13 @@
       <c r="B68" t="s">
         <v>225</v>
       </c>
-      <c r="C68" s="19" t="s">
+      <c r="C68" t="s">
         <v>243</v>
       </c>
-      <c r="D68" s="19" t="s">
+      <c r="D68" t="s">
         <v>244</v>
       </c>
-      <c r="E68" s="19" t="s">
+      <c r="E68" t="s">
         <v>530</v>
       </c>
     </row>
@@ -3685,13 +3682,13 @@
       <c r="B69" t="s">
         <v>224</v>
       </c>
-      <c r="C69" s="19" t="s">
+      <c r="C69" t="s">
         <v>243</v>
       </c>
-      <c r="D69" s="19" t="s">
+      <c r="D69" t="s">
         <v>244</v>
       </c>
-      <c r="E69" s="19" t="s">
+      <c r="E69" t="s">
         <v>530</v>
       </c>
     </row>
@@ -3702,14 +3699,14 @@
       <c r="B70" t="s">
         <v>201</v>
       </c>
-      <c r="C70" s="19" t="s">
+      <c r="C70" t="s">
         <v>243</v>
       </c>
-      <c r="D70" s="19" t="s">
+      <c r="D70" t="s">
         <v>244</v>
       </c>
-      <c r="E70" s="19" t="s">
-        <v>552</v>
+      <c r="E70" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
@@ -3719,14 +3716,14 @@
       <c r="B71" t="s">
         <v>508</v>
       </c>
-      <c r="C71" s="19" t="s">
+      <c r="C71" t="s">
         <v>243</v>
       </c>
-      <c r="D71" s="19" t="s">
+      <c r="D71" t="s">
         <v>244</v>
       </c>
-      <c r="E71" s="19" t="s">
-        <v>552</v>
+      <c r="E71" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.45">
@@ -3736,14 +3733,14 @@
       <c r="B72" t="s">
         <v>232</v>
       </c>
-      <c r="C72" s="19" t="s">
+      <c r="C72" t="s">
         <v>243</v>
       </c>
-      <c r="D72" s="19" t="s">
+      <c r="D72" t="s">
         <v>244</v>
       </c>
-      <c r="E72" s="19" t="s">
-        <v>552</v>
+      <c r="E72" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.45">
@@ -3753,14 +3750,14 @@
       <c r="B73" t="s">
         <v>207</v>
       </c>
-      <c r="C73" s="19" t="s">
+      <c r="C73" t="s">
         <v>243</v>
       </c>
-      <c r="D73" s="19" t="s">
+      <c r="D73" t="s">
         <v>244</v>
       </c>
-      <c r="E73" s="19" t="s">
-        <v>552</v>
+      <c r="E73" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.45">
@@ -3770,14 +3767,14 @@
       <c r="B74" t="s">
         <v>162</v>
       </c>
-      <c r="C74" s="19" t="s">
+      <c r="C74" t="s">
         <v>243</v>
       </c>
-      <c r="D74" s="19" t="s">
+      <c r="D74" t="s">
         <v>244</v>
       </c>
-      <c r="E74" s="19" t="s">
-        <v>552</v>
+      <c r="E74" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.45">
@@ -3787,14 +3784,14 @@
       <c r="B75" t="s">
         <v>204</v>
       </c>
-      <c r="C75" s="19" t="s">
+      <c r="C75" t="s">
         <v>243</v>
       </c>
-      <c r="D75" s="19" t="s">
+      <c r="D75" t="s">
         <v>244</v>
       </c>
-      <c r="E75" s="19" t="s">
-        <v>552</v>
+      <c r="E75" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.45">
@@ -3804,14 +3801,14 @@
       <c r="B76" t="s">
         <v>205</v>
       </c>
-      <c r="C76" s="19" t="s">
+      <c r="C76" t="s">
         <v>243</v>
       </c>
-      <c r="D76" s="19" t="s">
+      <c r="D76" t="s">
         <v>244</v>
       </c>
-      <c r="E76" s="19" t="s">
-        <v>552</v>
+      <c r="E76" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.45">
@@ -3821,14 +3818,14 @@
       <c r="B77" t="s">
         <v>230</v>
       </c>
-      <c r="C77" s="19" t="s">
+      <c r="C77" t="s">
         <v>243</v>
       </c>
-      <c r="D77" s="19" t="s">
+      <c r="D77" t="s">
         <v>244</v>
       </c>
-      <c r="E77" s="19" t="s">
-        <v>552</v>
+      <c r="E77" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.45">
@@ -3860,13 +3857,13 @@
       <c r="B80" t="s">
         <v>215</v>
       </c>
-      <c r="C80" s="19" t="s">
+      <c r="C80" t="s">
         <v>245</v>
       </c>
-      <c r="D80" s="19" t="s">
+      <c r="D80" t="s">
         <v>246</v>
       </c>
-      <c r="E80" s="19" t="s">
+      <c r="E80" t="s">
         <v>253</v>
       </c>
     </row>
@@ -3877,13 +3874,13 @@
       <c r="B81" t="s">
         <v>187</v>
       </c>
-      <c r="C81" s="19" t="s">
+      <c r="C81" t="s">
         <v>245</v>
       </c>
-      <c r="D81" s="19" t="s">
+      <c r="D81" t="s">
         <v>246</v>
       </c>
-      <c r="E81" s="19" t="s">
+      <c r="E81" t="s">
         <v>253</v>
       </c>
     </row>
@@ -3894,14 +3891,14 @@
       <c r="B82" t="s">
         <v>154</v>
       </c>
-      <c r="C82" s="19" t="s">
+      <c r="C82" t="s">
         <v>245</v>
       </c>
-      <c r="D82" s="19" t="s">
+      <c r="D82" t="s">
         <v>246</v>
       </c>
-      <c r="E82" s="19" t="s">
-        <v>553</v>
+      <c r="E82" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.45">
@@ -3911,14 +3908,14 @@
       <c r="B83" t="s">
         <v>231</v>
       </c>
-      <c r="C83" s="19" t="s">
+      <c r="C83" t="s">
         <v>245</v>
       </c>
-      <c r="D83" s="19" t="s">
+      <c r="D83" t="s">
         <v>246</v>
       </c>
-      <c r="E83" s="19" t="s">
-        <v>553</v>
+      <c r="E83" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.45">
@@ -3928,14 +3925,14 @@
       <c r="B84" t="s">
         <v>182</v>
       </c>
-      <c r="C84" s="19" t="s">
+      <c r="C84" t="s">
         <v>245</v>
       </c>
-      <c r="D84" s="19" t="s">
+      <c r="D84" t="s">
         <v>246</v>
       </c>
-      <c r="E84" s="19" t="s">
-        <v>553</v>
+      <c r="E84" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.45">
@@ -3945,14 +3942,14 @@
       <c r="B85" t="s">
         <v>144</v>
       </c>
-      <c r="C85" s="19" t="s">
+      <c r="C85" t="s">
         <v>245</v>
       </c>
-      <c r="D85" s="19" t="s">
+      <c r="D85" t="s">
         <v>246</v>
       </c>
-      <c r="E85" s="19" t="s">
-        <v>553</v>
+      <c r="E85" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.45">
@@ -3962,14 +3959,14 @@
       <c r="B86" t="s">
         <v>222</v>
       </c>
-      <c r="C86" s="19" t="s">
+      <c r="C86" t="s">
         <v>245</v>
       </c>
-      <c r="D86" s="19" t="s">
+      <c r="D86" t="s">
         <v>246</v>
       </c>
-      <c r="E86" s="19" t="s">
-        <v>553</v>
+      <c r="E86" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.45">
@@ -3979,14 +3976,14 @@
       <c r="B87" t="s">
         <v>155</v>
       </c>
-      <c r="C87" s="19" t="s">
+      <c r="C87" t="s">
         <v>245</v>
       </c>
-      <c r="D87" s="19" t="s">
+      <c r="D87" t="s">
         <v>246</v>
       </c>
-      <c r="E87" s="19" t="s">
-        <v>553</v>
+      <c r="E87" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.45">
@@ -3996,14 +3993,14 @@
       <c r="B88" t="s">
         <v>202</v>
       </c>
-      <c r="C88" s="19" t="s">
+      <c r="C88" t="s">
         <v>245</v>
       </c>
-      <c r="D88" s="19" t="s">
+      <c r="D88" t="s">
         <v>246</v>
       </c>
-      <c r="E88" s="19" t="s">
-        <v>553</v>
+      <c r="E88" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.45">
@@ -4013,13 +4010,13 @@
       <c r="B89" t="s">
         <v>196</v>
       </c>
-      <c r="C89" s="19" t="s">
+      <c r="C89" t="s">
         <v>255</v>
       </c>
-      <c r="D89" s="19" t="s">
+      <c r="D89" t="s">
         <v>256</v>
       </c>
-      <c r="E89" s="19" t="s">
+      <c r="E89" t="s">
         <v>531</v>
       </c>
     </row>
@@ -4030,13 +4027,13 @@
       <c r="B90" t="s">
         <v>180</v>
       </c>
-      <c r="C90" s="19" t="s">
+      <c r="C90" t="s">
         <v>255</v>
       </c>
-      <c r="D90" s="19" t="s">
+      <c r="D90" t="s">
         <v>256</v>
       </c>
-      <c r="E90" s="19" t="s">
+      <c r="E90" t="s">
         <v>531</v>
       </c>
     </row>
@@ -4047,14 +4044,14 @@
       <c r="B91" t="s">
         <v>210</v>
       </c>
-      <c r="C91" s="19" t="s">
+      <c r="C91" t="s">
         <v>255</v>
       </c>
-      <c r="D91" s="19" t="s">
+      <c r="D91" t="s">
         <v>256</v>
       </c>
-      <c r="E91" s="19" t="s">
-        <v>554</v>
+      <c r="E91" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.45">
@@ -4064,14 +4061,14 @@
       <c r="B92" t="s">
         <v>200</v>
       </c>
-      <c r="C92" s="19" t="s">
+      <c r="C92" t="s">
         <v>255</v>
       </c>
-      <c r="D92" s="19" t="s">
+      <c r="D92" t="s">
         <v>256</v>
       </c>
-      <c r="E92" s="19" t="s">
-        <v>554</v>
+      <c r="E92" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.45">
@@ -4081,14 +4078,14 @@
       <c r="B93" t="s">
         <v>149</v>
       </c>
-      <c r="C93" s="19" t="s">
+      <c r="C93" t="s">
         <v>255</v>
       </c>
-      <c r="D93" s="19" t="s">
+      <c r="D93" t="s">
         <v>256</v>
       </c>
-      <c r="E93" s="19" t="s">
-        <v>554</v>
+      <c r="E93" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.45">
@@ -4098,14 +4095,14 @@
       <c r="B94" t="s">
         <v>179</v>
       </c>
-      <c r="C94" s="19" t="s">
+      <c r="C94" t="s">
         <v>255</v>
       </c>
-      <c r="D94" s="19" t="s">
+      <c r="D94" t="s">
         <v>256</v>
       </c>
-      <c r="E94" s="19" t="s">
-        <v>554</v>
+      <c r="E94" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.45">
@@ -4115,14 +4112,14 @@
       <c r="B95" t="s">
         <v>219</v>
       </c>
-      <c r="C95" s="19" t="s">
+      <c r="C95" t="s">
         <v>255</v>
       </c>
-      <c r="D95" s="19" t="s">
+      <c r="D95" t="s">
         <v>256</v>
       </c>
-      <c r="E95" s="19" t="s">
-        <v>554</v>
+      <c r="E95" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.45">
@@ -4132,14 +4129,14 @@
       <c r="B96" t="s">
         <v>175</v>
       </c>
-      <c r="C96" s="19" t="s">
+      <c r="C96" t="s">
         <v>255</v>
       </c>
-      <c r="D96" s="19" t="s">
+      <c r="D96" t="s">
         <v>256</v>
       </c>
-      <c r="E96" s="19" t="s">
-        <v>554</v>
+      <c r="E96" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.45">
@@ -4149,14 +4146,14 @@
       <c r="B97" t="s">
         <v>181</v>
       </c>
-      <c r="C97" s="19" t="s">
+      <c r="C97" t="s">
         <v>255</v>
       </c>
-      <c r="D97" s="19" t="s">
+      <c r="D97" t="s">
         <v>256</v>
       </c>
-      <c r="E97" s="19" t="s">
-        <v>554</v>
+      <c r="E97" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.45">
@@ -4166,14 +4163,14 @@
       <c r="B98" t="s">
         <v>220</v>
       </c>
-      <c r="C98" s="19" t="s">
+      <c r="C98" t="s">
         <v>255</v>
       </c>
-      <c r="D98" s="19" t="s">
+      <c r="D98" t="s">
         <v>256</v>
       </c>
-      <c r="E98" s="19" t="s">
-        <v>554</v>
+      <c r="E98" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.45">
@@ -4205,13 +4202,13 @@
       <c r="B101" t="s">
         <v>203</v>
       </c>
-      <c r="C101" s="19" t="s">
+      <c r="C101" t="s">
         <v>258</v>
       </c>
-      <c r="D101" s="19" t="s">
+      <c r="D101" t="s">
         <v>257</v>
       </c>
-      <c r="E101" s="19" t="s">
+      <c r="E101" t="s">
         <v>254</v>
       </c>
     </row>
@@ -4222,13 +4219,13 @@
       <c r="B102" t="s">
         <v>173</v>
       </c>
-      <c r="C102" s="19" t="s">
+      <c r="C102" t="s">
         <v>258</v>
       </c>
-      <c r="D102" s="19" t="s">
+      <c r="D102" t="s">
         <v>257</v>
       </c>
-      <c r="E102" s="19" t="s">
+      <c r="E102" t="s">
         <v>254</v>
       </c>
     </row>
@@ -4239,14 +4236,14 @@
       <c r="B103" t="s">
         <v>228</v>
       </c>
-      <c r="C103" s="19" t="s">
+      <c r="C103" t="s">
         <v>258</v>
       </c>
-      <c r="D103" s="19" t="s">
+      <c r="D103" t="s">
         <v>257</v>
       </c>
-      <c r="E103" s="19" t="s">
-        <v>555</v>
+      <c r="E103" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.45">
@@ -4256,14 +4253,14 @@
       <c r="B104" t="s">
         <v>170</v>
       </c>
-      <c r="C104" s="19" t="s">
+      <c r="C104" t="s">
         <v>258</v>
       </c>
-      <c r="D104" s="19" t="s">
+      <c r="D104" t="s">
         <v>257</v>
       </c>
-      <c r="E104" s="19" t="s">
-        <v>555</v>
+      <c r="E104" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.45">
@@ -4273,14 +4270,14 @@
       <c r="B105" t="s">
         <v>153</v>
       </c>
-      <c r="C105" s="19" t="s">
+      <c r="C105" t="s">
         <v>258</v>
       </c>
-      <c r="D105" s="19" t="s">
+      <c r="D105" t="s">
         <v>257</v>
       </c>
-      <c r="E105" s="19" t="s">
-        <v>555</v>
+      <c r="E105" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.45">
@@ -4290,14 +4287,14 @@
       <c r="B106" t="s">
         <v>150</v>
       </c>
-      <c r="C106" s="19" t="s">
+      <c r="C106" t="s">
         <v>258</v>
       </c>
-      <c r="D106" s="19" t="s">
+      <c r="D106" t="s">
         <v>257</v>
       </c>
-      <c r="E106" s="19" t="s">
-        <v>555</v>
+      <c r="E106" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.45">
@@ -4307,14 +4304,14 @@
       <c r="B107" t="s">
         <v>185</v>
       </c>
-      <c r="C107" s="19" t="s">
+      <c r="C107" t="s">
         <v>258</v>
       </c>
-      <c r="D107" s="19" t="s">
+      <c r="D107" t="s">
         <v>257</v>
       </c>
-      <c r="E107" s="19" t="s">
-        <v>555</v>
+      <c r="E107" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.45">
@@ -4324,14 +4321,14 @@
       <c r="B108" t="s">
         <v>165</v>
       </c>
-      <c r="C108" s="19" t="s">
+      <c r="C108" t="s">
         <v>258</v>
       </c>
-      <c r="D108" s="19" t="s">
+      <c r="D108" t="s">
         <v>257</v>
       </c>
-      <c r="E108" s="19" t="s">
-        <v>555</v>
+      <c r="E108" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.45">
@@ -4341,14 +4338,14 @@
       <c r="B109" t="s">
         <v>216</v>
       </c>
-      <c r="C109" s="19" t="s">
+      <c r="C109" t="s">
         <v>258</v>
       </c>
-      <c r="D109" s="19" t="s">
+      <c r="D109" t="s">
         <v>257</v>
       </c>
-      <c r="E109" s="19" t="s">
-        <v>555</v>
+      <c r="E109" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.45">
@@ -4358,14 +4355,14 @@
       <c r="B110" t="s">
         <v>192</v>
       </c>
-      <c r="C110" s="19" t="s">
+      <c r="C110" t="s">
         <v>258</v>
       </c>
-      <c r="D110" s="19" t="s">
+      <c r="D110" t="s">
         <v>257</v>
       </c>
-      <c r="E110" s="19" t="s">
-        <v>555</v>
+      <c r="E110" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.45">
@@ -4375,14 +4372,14 @@
       <c r="B111" t="s">
         <v>151</v>
       </c>
-      <c r="C111" s="19" t="s">
+      <c r="C111" t="s">
         <v>258</v>
       </c>
-      <c r="D111" s="19" t="s">
+      <c r="D111" t="s">
         <v>257</v>
       </c>
-      <c r="E111" s="19" t="s">
-        <v>555</v>
+      <c r="E111" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.45">
@@ -4392,14 +4389,14 @@
       <c r="B112" t="s">
         <v>509</v>
       </c>
-      <c r="C112" s="19" t="s">
+      <c r="C112" t="s">
         <v>258</v>
       </c>
-      <c r="D112" s="19" t="s">
+      <c r="D112" t="s">
         <v>257</v>
       </c>
-      <c r="E112" s="19" t="s">
-        <v>555</v>
+      <c r="E112" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.45">
@@ -4409,14 +4406,14 @@
       <c r="B113" t="s">
         <v>177</v>
       </c>
-      <c r="C113" s="19" t="s">
+      <c r="C113" t="s">
         <v>258</v>
       </c>
-      <c r="D113" s="19" t="s">
+      <c r="D113" t="s">
         <v>257</v>
       </c>
-      <c r="E113" s="19" t="s">
-        <v>555</v>
+      <c r="E113" t="s">
+        <v>554</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.45">
@@ -4426,13 +4423,13 @@
       <c r="B114" t="s">
         <v>233</v>
       </c>
-      <c r="C114" s="19" t="s">
+      <c r="C114" t="s">
         <v>249</v>
       </c>
-      <c r="D114" s="19" t="s">
+      <c r="D114" t="s">
         <v>250</v>
       </c>
-      <c r="E114" s="19" t="s">
+      <c r="E114" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4443,13 +4440,13 @@
       <c r="B115" t="s">
         <v>206</v>
       </c>
-      <c r="C115" s="19" t="s">
+      <c r="C115" t="s">
         <v>249</v>
       </c>
-      <c r="D115" s="19" t="s">
+      <c r="D115" t="s">
         <v>250</v>
       </c>
-      <c r="E115" s="19" t="s">
+      <c r="E115" t="s">
         <v>251</v>
       </c>
     </row>
@@ -4460,14 +4457,14 @@
       <c r="B116" t="s">
         <v>194</v>
       </c>
-      <c r="C116" s="19" t="s">
+      <c r="C116" t="s">
         <v>249</v>
       </c>
-      <c r="D116" s="19" t="s">
+      <c r="D116" t="s">
         <v>250</v>
       </c>
-      <c r="E116" s="19" t="s">
-        <v>556</v>
+      <c r="E116" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.45">
@@ -4477,14 +4474,14 @@
       <c r="B117" t="s">
         <v>178</v>
       </c>
-      <c r="C117" s="19" t="s">
+      <c r="C117" t="s">
         <v>249</v>
       </c>
-      <c r="D117" s="19" t="s">
+      <c r="D117" t="s">
         <v>250</v>
       </c>
-      <c r="E117" s="19" t="s">
-        <v>556</v>
+      <c r="E117" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.45">
@@ -4494,14 +4491,14 @@
       <c r="B118" t="s">
         <v>223</v>
       </c>
-      <c r="C118" s="19" t="s">
+      <c r="C118" t="s">
         <v>249</v>
       </c>
-      <c r="D118" s="19" t="s">
+      <c r="D118" t="s">
         <v>250</v>
       </c>
-      <c r="E118" s="19" t="s">
-        <v>556</v>
+      <c r="E118" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.45">
@@ -4511,14 +4508,14 @@
       <c r="B119" t="s">
         <v>143</v>
       </c>
-      <c r="C119" s="19" t="s">
+      <c r="C119" t="s">
         <v>249</v>
       </c>
-      <c r="D119" s="19" t="s">
+      <c r="D119" t="s">
         <v>250</v>
       </c>
-      <c r="E119" s="19" t="s">
-        <v>556</v>
+      <c r="E119" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.45">
@@ -4528,14 +4525,14 @@
       <c r="B120" t="s">
         <v>169</v>
       </c>
-      <c r="C120" s="19" t="s">
+      <c r="C120" t="s">
         <v>249</v>
       </c>
-      <c r="D120" s="19" t="s">
+      <c r="D120" t="s">
         <v>250</v>
       </c>
-      <c r="E120" s="19" t="s">
-        <v>556</v>
+      <c r="E120" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.45">
@@ -4545,14 +4542,14 @@
       <c r="B121" t="s">
         <v>166</v>
       </c>
-      <c r="C121" s="19" t="s">
+      <c r="C121" t="s">
         <v>249</v>
       </c>
-      <c r="D121" s="19" t="s">
+      <c r="D121" t="s">
         <v>250</v>
       </c>
-      <c r="E121" s="19" t="s">
-        <v>556</v>
+      <c r="E121" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.45">
@@ -4562,14 +4559,14 @@
       <c r="B122" t="s">
         <v>186</v>
       </c>
-      <c r="C122" s="19" t="s">
+      <c r="C122" t="s">
         <v>249</v>
       </c>
-      <c r="D122" s="19" t="s">
+      <c r="D122" t="s">
         <v>250</v>
       </c>
-      <c r="E122" s="19" t="s">
-        <v>556</v>
+      <c r="E122" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.45">
@@ -4579,14 +4576,14 @@
       <c r="B123" t="s">
         <v>199</v>
       </c>
-      <c r="C123" s="19" t="s">
+      <c r="C123" t="s">
         <v>249</v>
       </c>
-      <c r="D123" s="19" t="s">
+      <c r="D123" t="s">
         <v>250</v>
       </c>
-      <c r="E123" s="19" t="s">
-        <v>556</v>
+      <c r="E123" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.45">
@@ -4596,14 +4593,14 @@
       <c r="B124" t="s">
         <v>157</v>
       </c>
-      <c r="C124" s="19" t="s">
+      <c r="C124" t="s">
         <v>249</v>
       </c>
-      <c r="D124" s="19" t="s">
+      <c r="D124" t="s">
         <v>250</v>
       </c>
-      <c r="E124" s="19" t="s">
-        <v>556</v>
+      <c r="E124" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.45">
@@ -4613,14 +4610,14 @@
       <c r="B125" t="s">
         <v>158</v>
       </c>
-      <c r="C125" s="19" t="s">
+      <c r="C125" t="s">
         <v>249</v>
       </c>
-      <c r="D125" s="19" t="s">
+      <c r="D125" t="s">
         <v>250</v>
       </c>
-      <c r="E125" s="19" t="s">
-        <v>556</v>
+      <c r="E125" t="s">
+        <v>555</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.45">
@@ -4652,13 +4649,13 @@
       <c r="B128" t="s">
         <v>197</v>
       </c>
-      <c r="C128" s="19" t="s">
+      <c r="C128" t="s">
         <v>261</v>
       </c>
-      <c r="D128" s="19" t="s">
+      <c r="D128" t="s">
         <v>260</v>
       </c>
-      <c r="E128" s="19" t="s">
+      <c r="E128" t="s">
         <v>259</v>
       </c>
     </row>
@@ -4669,13 +4666,13 @@
       <c r="B129" t="s">
         <v>211</v>
       </c>
-      <c r="C129" s="19" t="s">
+      <c r="C129" t="s">
         <v>261</v>
       </c>
-      <c r="D129" s="19" t="s">
+      <c r="D129" t="s">
         <v>260</v>
       </c>
-      <c r="E129" s="19" t="s">
+      <c r="E129" t="s">
         <v>259</v>
       </c>
     </row>
@@ -4686,14 +4683,14 @@
       <c r="B130" t="s">
         <v>184</v>
       </c>
-      <c r="C130" s="19" t="s">
+      <c r="C130" t="s">
         <v>261</v>
       </c>
-      <c r="D130" s="19" t="s">
+      <c r="D130" t="s">
         <v>260</v>
       </c>
-      <c r="E130" s="19" t="s">
-        <v>557</v>
+      <c r="E130" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.45">
@@ -4703,14 +4700,14 @@
       <c r="B131" t="s">
         <v>229</v>
       </c>
-      <c r="C131" s="19" t="s">
+      <c r="C131" t="s">
         <v>261</v>
       </c>
-      <c r="D131" s="19" t="s">
+      <c r="D131" t="s">
         <v>260</v>
       </c>
-      <c r="E131" s="19" t="s">
-        <v>557</v>
+      <c r="E131" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.45">
@@ -4720,14 +4717,14 @@
       <c r="B132" t="s">
         <v>172</v>
       </c>
-      <c r="C132" s="19" t="s">
+      <c r="C132" t="s">
         <v>261</v>
       </c>
-      <c r="D132" s="19" t="s">
+      <c r="D132" t="s">
         <v>260</v>
       </c>
-      <c r="E132" s="19" t="s">
-        <v>557</v>
+      <c r="E132" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.45">
@@ -4737,14 +4734,14 @@
       <c r="B133" t="s">
         <v>221</v>
       </c>
-      <c r="C133" s="19" t="s">
+      <c r="C133" t="s">
         <v>261</v>
       </c>
-      <c r="D133" s="19" t="s">
+      <c r="D133" t="s">
         <v>260</v>
       </c>
-      <c r="E133" s="19" t="s">
-        <v>557</v>
+      <c r="E133" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.45">
@@ -4754,14 +4751,14 @@
       <c r="B134" t="s">
         <v>218</v>
       </c>
-      <c r="C134" s="19" t="s">
+      <c r="C134" t="s">
         <v>261</v>
       </c>
-      <c r="D134" s="19" t="s">
+      <c r="D134" t="s">
         <v>260</v>
       </c>
-      <c r="E134" s="19" t="s">
-        <v>557</v>
+      <c r="E134" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.45">
@@ -4771,14 +4768,14 @@
       <c r="B135" t="s">
         <v>174</v>
       </c>
-      <c r="C135" s="19" t="s">
+      <c r="C135" t="s">
         <v>261</v>
       </c>
-      <c r="D135" s="19" t="s">
+      <c r="D135" t="s">
         <v>260</v>
       </c>
-      <c r="E135" s="19" t="s">
-        <v>557</v>
+      <c r="E135" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.45">
@@ -4788,14 +4785,14 @@
       <c r="B136" t="s">
         <v>209</v>
       </c>
-      <c r="C136" s="19" t="s">
+      <c r="C136" t="s">
         <v>261</v>
       </c>
-      <c r="D136" s="19" t="s">
+      <c r="D136" t="s">
         <v>260</v>
       </c>
-      <c r="E136" s="19" t="s">
-        <v>557</v>
+      <c r="E136" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.45">
@@ -4805,14 +4802,14 @@
       <c r="B137" t="s">
         <v>183</v>
       </c>
-      <c r="C137" s="19" t="s">
+      <c r="C137" t="s">
         <v>261</v>
       </c>
-      <c r="D137" s="19" t="s">
+      <c r="D137" t="s">
         <v>260</v>
       </c>
-      <c r="E137" s="19" t="s">
-        <v>557</v>
+      <c r="E137" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.45">
@@ -4822,14 +4819,14 @@
       <c r="B138" t="s">
         <v>160</v>
       </c>
-      <c r="C138" s="19" t="s">
+      <c r="C138" t="s">
         <v>261</v>
       </c>
-      <c r="D138" s="19" t="s">
+      <c r="D138" t="s">
         <v>260</v>
       </c>
-      <c r="E138" s="19" t="s">
-        <v>557</v>
+      <c r="E138" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.45">
@@ -4839,14 +4836,14 @@
       <c r="B139" t="s">
         <v>171</v>
       </c>
-      <c r="C139" s="19" t="s">
+      <c r="C139" t="s">
         <v>261</v>
       </c>
-      <c r="D139" s="19" t="s">
+      <c r="D139" t="s">
         <v>260</v>
       </c>
-      <c r="E139" s="19" t="s">
-        <v>557</v>
+      <c r="E139" t="s">
+        <v>556</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.45">
@@ -4868,19 +4865,19 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
+        <v>541</v>
+      </c>
+      <c r="B142" t="s">
+        <v>539</v>
+      </c>
+      <c r="C142" t="s">
         <v>542</v>
       </c>
-      <c r="B142" t="s">
-        <v>540</v>
-      </c>
-      <c r="C142" t="s">
+      <c r="D142" t="s">
         <v>543</v>
       </c>
-      <c r="D142" t="s">
-        <v>544</v>
-      </c>
       <c r="E142" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
   </sheetData>
@@ -5711,7 +5708,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B30">
         <v>70</v>
@@ -11955,7 +11952,7 @@
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A253" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B253">
         <v>1</v>
@@ -11975,10 +11972,10 @@
         <v>1</v>
       </c>
       <c r="G253" t="s">
+        <v>540</v>
+      </c>
+      <c r="H253" t="s">
         <v>541</v>
-      </c>
-      <c r="H253" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.45">
@@ -12107,7 +12104,7 @@
         <v>72</v>
       </c>
       <c r="E258">
-        <f t="shared" ref="E258:E321" si="8">SUM(B258:D258)</f>
+        <f t="shared" ref="E258:E261" si="8">SUM(B258:D258)</f>
         <v>201</v>
       </c>
       <c r="F258">
@@ -12302,7 +12299,7 @@
         <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -12928,12 +12925,12 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.45">

</xml_diff>